<commit_message>
Lista Mestra E01: preenche CONTEÚDO com o TÍTULO do carimbo dos PDFs
</commit_message>
<xml_diff>
--- a/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
+++ b/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="77">
   <si>
     <t>LISTA MESTRA DE PROJETOS</t>
   </si>
@@ -61,103 +61,187 @@
     <t>A1</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO E DETALHES</t>
+  </si>
+  <si>
     <t>EMISSÃO INICIAL</t>
   </si>
   <si>
     <t>LOGSLS-ARQ-101-PE-IMP_ROT</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO ROTA ACESSÍVEL E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-102-PE-IMP_CERC</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO CERCAMENTO E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-103-PE-IMP_DEF_VID</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO DEFENSA, LINHA DE VIDA E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-104-PE-IMP_RAIO</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO RAIOS DE GIRO</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-105-PE-IMP_PASS</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO PASSEIOS</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-106-PE-IMP_PORT</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO PORTÕES DE ACESSO</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-107-PE-IMP_IRRIG</t>
   </si>
   <si>
+    <t>IMPLANTAÇÃO IRRIGAÇÃO</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-200-PE-G01_1ºPAV_2ºPAV</t>
   </si>
   <si>
     <t>A0+</t>
   </si>
   <si>
+    <t>GALPÃO PLANTAS 1º PAVIMENTO E MEZANINO</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-201-PE-G01_COR_COB</t>
   </si>
   <si>
+    <t>GALPÃO CORTES, PLANTA DE COBERTURA E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-202-PE-G01_FAC</t>
   </si>
   <si>
+    <t>GALPÃO FACHADAS, PERSPECTIVA E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-203-PE-G01_LAY</t>
   </si>
   <si>
+    <t>GALPÃO PLANTA, CORTE LAYOUT PORTA PALLETS E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-204-PE-G01_DET1_1A_PAV1_MEZ</t>
   </si>
   <si>
     <t>A1++</t>
   </si>
   <si>
+    <t>GALPÃO DETALHE 1 E 1A - ACESSO CENTRAL - PLANTAS 1º PAVIMENTO E MEZANINO - PERSPECTIVAS E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-205-PE-G01_DET1_1A_COR_FAC</t>
   </si>
   <si>
     <t>A0</t>
   </si>
   <si>
+    <t>GALPÃO DETALHE 1 E 1A - ACESSO CENTRAL - CORTES, FACHADA E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-206-PE-G01_DET2_PAV1_MEZ</t>
   </si>
   <si>
+    <t>GALPÃO DETALHE 2 - ACESSO LATERAL - PLANTAS 1º PAVIMENTO E MEZANINO, PERSPECTIVAS E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-207-PE-G01_DET2_COR_FAC</t>
   </si>
   <si>
+    <t>GALPÃO DETALHE 2- ACESSO LATERAL - CORTES, FACHADA E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-300-PE-PORT_PAV1_LAY_COB_COR</t>
   </si>
   <si>
+    <t>PORTARIA E APOIO CAMINHONEIRO PLANTA DE ALVENARIAS, LAYOUT, CORTES E PLANTA DE COBERTURA</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-301-PE-PORT_COR_FAC</t>
   </si>
   <si>
     <t>A1+</t>
   </si>
   <si>
+    <t>PORTARIA E APOIO CAMINHONEIRO CORTE, FACHADAS, DETALHES E PERSPECTIVA</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-302-PE-PORT-FOR</t>
   </si>
   <si>
     <t>A2</t>
   </si>
   <si>
+    <t>PORTARIA / APOIO CAMINHONEIRO PLANTA DE FORRO</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-303-PE-REST-VEST-LAZ_PAV1_PAV2_COB</t>
   </si>
   <si>
+    <t>RESTAURANTE E VESTIÁRIO PLANTAS 1º E 2º PAVIMENTOS, PLANTA DE COBERTURA E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-304-PE-REST-VEST_COR_FAC</t>
   </si>
   <si>
+    <t>RESTAURANTE E VESTIÁRIO PLANTAS LAYOUT, CORTES, FACHADAS E DETALHES</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-305-PE-REST-VEST-LAZ_FOR</t>
   </si>
   <si>
+    <t>RESTAURANTE E VESTIÁRIO PLANTA DE FORRO</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-306-PE-BOM_GER</t>
   </si>
   <si>
+    <t>CASA DE BOMBAS PLANTA, CORTES, FACHADAS, PLANTA DE COBERTURA, PERSPECTIVA E DETALHE</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-307-PE-ARS_GER</t>
   </si>
   <si>
+    <t>ABRIGO DE RESÍDUOS SÓLIDOS PLANTA, CORTES, FACHADAS, PLANTA DE COBERTURA, PERSPECTIVA E DETALHE</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-308-PE-GÁS_GER</t>
   </si>
   <si>
+    <t>CENTRAL DE GÁS PLANTA, CORTES, FACHADAS, PLANTA DE COBERTURA, PERSPECTIVA E DETALHE</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-309-PE-MED_GER</t>
   </si>
   <si>
+    <t>CABINE DE MEDIÇÃO PLANTA, CORTES, FACHADAS, PLANTA DE COBERTURA, PERSPECTIVA E DETALHE</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-310-PE-SUB 1 3 4 _GER</t>
   </si>
   <si>
+    <t>SUBESTAÇÃO 1,3 e 4 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACAHDAS, DETALHE E PERSPECTIVA</t>
+  </si>
+  <si>
     <t>LOGSLS-ARQ-311-PE-SUB2_GER</t>
+  </si>
+  <si>
+    <t>SUBESTAÇÃO 2 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACAHDAS, DETALHE E PERSPECTIVA</t>
   </si>
 </sst>
 </file>
@@ -918,15 +1002,15 @@
         <v>15</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" s="11">
         <v>0</v>
@@ -938,15 +1022,15 @@
         <v>15</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="11">
         <v>0</v>
@@ -958,15 +1042,15 @@
         <v>15</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B11" s="11">
         <v>0</v>
@@ -978,15 +1062,15 @@
         <v>15</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B12" s="11">
         <v>0</v>
@@ -998,15 +1082,15 @@
         <v>15</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B13" s="11">
         <v>0</v>
@@ -1018,15 +1102,15 @@
         <v>15</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B14" s="11">
         <v>0</v>
@@ -1038,15 +1122,15 @@
         <v>15</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B15" s="11">
         <v>0</v>
@@ -1058,15 +1142,15 @@
         <v>15</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B16" s="11">
         <v>0</v>
@@ -1075,18 +1159,18 @@
         <v>46093</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B17" s="11">
         <v>0</v>
@@ -1095,18 +1179,18 @@
         <v>46093</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B18" s="11">
         <v>0</v>
@@ -1115,18 +1199,18 @@
         <v>46093</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B19" s="11">
         <v>0</v>
@@ -1135,18 +1219,18 @@
         <v>46093</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B20" s="11">
         <v>0</v>
@@ -1155,18 +1239,18 @@
         <v>46093</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="B21" s="11">
         <v>0</v>
@@ -1175,18 +1259,18 @@
         <v>46093</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="B22" s="11">
         <v>0</v>
@@ -1198,15 +1282,15 @@
         <v>15</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="B23" s="11">
         <v>0</v>
@@ -1215,18 +1299,18 @@
         <v>46093</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="B24" s="11">
         <v>0</v>
@@ -1235,54 +1319,54 @@
         <v>46093</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="12">
         <v>46093</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>2</v>
+        <v>55</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="12">
         <v>46093</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="B27" s="11">
         <v>0</v>
@@ -1291,18 +1375,18 @@
         <v>46093</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B28" s="11">
         <v>0</v>
@@ -1311,18 +1395,18 @@
         <v>46093</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B29" s="11">
         <v>0</v>
@@ -1331,18 +1415,18 @@
         <v>46093</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="B30" s="11">
         <v>0</v>
@@ -1354,15 +1438,15 @@
         <v>15</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>2</v>
+        <v>66</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="B31" s="11">
         <v>0</v>
@@ -1374,15 +1458,15 @@
         <v>15</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="B32" s="11">
         <v>0</v>
@@ -1394,15 +1478,15 @@
         <v>15</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>2</v>
+        <v>70</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>46</v>
+        <v>71</v>
       </c>
       <c r="B33" s="11">
         <v>0</v>
@@ -1414,15 +1498,15 @@
         <v>15</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" ht="45" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="B34" s="11">
         <v>0</v>
@@ -1434,15 +1518,15 @@
         <v>15</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" ht="45" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B35" s="16">
         <v>0</v>
@@ -1454,10 +1538,10 @@
         <v>15</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>2</v>
+        <v>76</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lista Mestra E01: corrige typo FACAHDAS->FACHADAS na coluna CONTEÚDO
</commit_message>
<xml_diff>
--- a/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
+++ b/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
@@ -235,13 +235,13 @@
     <t>LOGSLS-ARQ-310-PE-SUB 1 3 4 _GER</t>
   </si>
   <si>
-    <t>SUBESTAÇÃO 1,3 e 4 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACAHDAS, DETALHE E PERSPECTIVA</t>
+    <t>SUBESTAÇÃO 1,3 e 4 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACHADAS, DETALHE E PERSPECTIVA</t>
   </si>
   <si>
     <t>LOGSLS-ARQ-311-PE-SUB2_GER</t>
   </si>
   <si>
-    <t>SUBESTAÇÃO 2 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACAHDAS, DETALHE E PERSPECTIVA</t>
+    <t>SUBESTAÇÃO 2 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACHADAS, DETALHE E PERSPECTIVA</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
TÍTULO: normaliza typos e espaçamento (app + Lista Mestra E01)
</commit_message>
<xml_diff>
--- a/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
+++ b/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
@@ -163,7 +163,7 @@
     <t>LOGSLS-ARQ-207-PE-G01_DET2_COR_FAC</t>
   </si>
   <si>
-    <t>GALPÃO DETALHE 2- ACESSO LATERAL - CORTES, FACHADA E DETALHES</t>
+    <t>GALPÃO DETALHE 2 - ACESSO LATERAL - CORTES, FACHADA E DETALHES</t>
   </si>
   <si>
     <t>LOGSLS-ARQ-300-PE-PORT_PAV1_LAY_COB_COR</t>
@@ -235,7 +235,7 @@
     <t>LOGSLS-ARQ-310-PE-SUB 1 3 4 _GER</t>
   </si>
   <si>
-    <t>SUBESTAÇÃO 1,3 e 4 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACHADAS, DETALHE E PERSPECTIVA</t>
+    <t>SUBESTAÇÃO 1, 3 e 4 - SALA DE QUADROS E TRANSFORMADOR PLANTA, PLANTA DE COBERTURA, CORTES, FACHADAS, DETALHE E PERSPECTIVA</t>
   </si>
   <si>
     <t>LOGSLS-ARQ-311-PE-SUB2_GER</t>

</xml_diff>

<commit_message>
Linhas de dados com preenchimento cinza #BFBFBF e altura automatica do ENDERECO
</commit_message>
<xml_diff>
--- a/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
+++ b/entregas/LOGSLS-ARQ-001-PL-LM_E01.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="78">
   <si>
     <t>LISTA MESTRA DE PROJETOS</t>
   </si>
@@ -19,10 +19,13 @@
     <t>OBRA</t>
   </si>
   <si>
-    <t/>
+    <t>LOG SÃO LUÍS</t>
   </si>
   <si>
     <t>ENDEREÇO</t>
+  </si>
+  <si>
+    <t>DISTRITO DE SÃO JOAQUIM DO BACANGA - KM 11, BR-135, GLEBA BACABAL - À MARGEM ESQUERDA DA RODOVIA SÃO LUÍS-TERESINA - SÃO LUÍS/MA</t>
   </si>
   <si>
     <t>PROJETO</t>
@@ -283,7 +286,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -293,6 +296,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBFBFBF"/>
       </patternFill>
     </fill>
   </fills>
@@ -433,34 +441,34 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -920,7 +928,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" ht="68" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3"/>
       <c r="C3"/>
@@ -929,7 +937,7 @@
         <v>3</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -938,10 +946,10 @@
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -950,10 +958,10 @@
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -962,7 +970,7 @@
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" s="8">
         <v>46093</v>
@@ -970,27 +978,27 @@
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>8</v>
-      </c>
       <c r="D7" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" s="11">
         <v>0</v>
@@ -999,18 +1007,18 @@
         <v>46093</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="11">
         <v>0</v>
@@ -1019,18 +1027,18 @@
         <v>46093</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="11">
         <v>0</v>
@@ -1039,18 +1047,18 @@
         <v>46093</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="11">
         <v>0</v>
@@ -1059,18 +1067,18 @@
         <v>46093</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="11">
         <v>0</v>
@@ -1079,18 +1087,18 @@
         <v>46093</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="11">
         <v>0</v>
@@ -1099,18 +1107,18 @@
         <v>46093</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B14" s="11">
         <v>0</v>
@@ -1119,18 +1127,18 @@
         <v>46093</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="11">
         <v>0</v>
@@ -1139,18 +1147,18 @@
         <v>46093</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" s="11">
         <v>0</v>
@@ -1159,18 +1167,18 @@
         <v>46093</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" s="11">
         <v>0</v>
@@ -1179,18 +1187,18 @@
         <v>46093</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="11">
         <v>0</v>
@@ -1199,18 +1207,18 @@
         <v>46093</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" s="11">
         <v>0</v>
@@ -1219,18 +1227,18 @@
         <v>46093</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B20" s="11">
         <v>0</v>
@@ -1239,18 +1247,18 @@
         <v>46093</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" s="11">
         <v>0</v>
@@ -1259,18 +1267,18 @@
         <v>46093</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22" s="11">
         <v>0</v>
@@ -1279,18 +1287,18 @@
         <v>46093</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="11">
         <v>0</v>
@@ -1299,18 +1307,18 @@
         <v>46093</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B24" s="11">
         <v>0</v>
@@ -1319,54 +1327,54 @@
         <v>46093</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="12">
         <v>46093</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="12">
         <v>46093</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B27" s="11">
         <v>0</v>
@@ -1375,18 +1383,18 @@
         <v>46093</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B28" s="11">
         <v>0</v>
@@ -1395,18 +1403,18 @@
         <v>46093</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B29" s="11">
         <v>0</v>
@@ -1415,18 +1423,18 @@
         <v>46093</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B30" s="11">
         <v>0</v>
@@ -1435,18 +1443,18 @@
         <v>46093</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B31" s="11">
         <v>0</v>
@@ -1455,18 +1463,18 @@
         <v>46093</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B32" s="11">
         <v>0</v>
@@ -1475,18 +1483,18 @@
         <v>46093</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B33" s="11">
         <v>0</v>
@@ -1495,18 +1503,18 @@
         <v>46093</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" ht="45" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B34" s="11">
         <v>0</v>
@@ -1515,18 +1523,18 @@
         <v>46093</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B35" s="16">
         <v>0</v>
@@ -1535,13 +1543,13 @@
         <v>46093</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>